<commit_message>
updated measurement table template
</commit_message>
<xml_diff>
--- a/2_Assessments/Measurement_Table_Template.xlsx
+++ b/2_Assessments/Measurement_Table_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D63A224-374C-2649-BA00-C92966CE6B24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4C153F0-9DA7-8D4E-A103-F8AF1B04B404}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-37840" yWindow="-5220" windowWidth="34640" windowHeight="23140" xr2:uid="{4F5E00DF-9948-D646-B558-8B1F78610CF0}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="28800" windowHeight="16220" xr2:uid="{4F5E00DF-9948-D646-B558-8B1F78610CF0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="62">
   <si>
     <t>Voltages</t>
   </si>
@@ -39,9 +39,6 @@
     <t>Voltage at +3V3 (VD)</t>
   </si>
   <si>
-    <t>Expexted</t>
-  </si>
-  <si>
     <t>Min</t>
   </si>
   <si>
@@ -87,9 +84,6 @@
     <t>Current on Power in at 5V, 3V0 unconnected</t>
   </si>
   <si>
-    <t>Current Ripple</t>
-  </si>
-  <si>
     <t>Microphone</t>
   </si>
   <si>
@@ -108,9 +102,6 @@
     <t>Reference Voltage U4</t>
   </si>
   <si>
-    <t>Reference Voltage In- (Offset)</t>
-  </si>
-  <si>
     <t>Line</t>
   </si>
   <si>
@@ -189,7 +180,43 @@
     <t>Note how you define Min/Max for each measurement</t>
   </si>
   <si>
-    <t>all other measurements are mandatory, but required to demonstrate</t>
+    <t>&lt;5</t>
+  </si>
+  <si>
+    <t>orange = don't need to fill up</t>
+  </si>
+  <si>
+    <t>&lt;180 mA</t>
+  </si>
+  <si>
+    <t>&lt;160 mA</t>
+  </si>
+  <si>
+    <t>50 mV</t>
+  </si>
+  <si>
+    <t>2.5 V</t>
+  </si>
+  <si>
+    <t>&gt;300 mV</t>
+  </si>
+  <si>
+    <t>&gt;2 V</t>
+  </si>
+  <si>
+    <t>Generate a 500 mVpp 1 kHz signal and measure the amplitude at Line Input</t>
+  </si>
+  <si>
+    <t>500 mVpp</t>
+  </si>
+  <si>
+    <t>all other measuremtents are mandatory, but not required to demonstrate</t>
+  </si>
+  <si>
+    <t>Current Ripple on Power in at 5 V</t>
+  </si>
+  <si>
+    <t>Expected</t>
   </si>
 </sst>
 </file>
@@ -219,7 +246,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -238,6 +265,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -251,16 +284,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -276,7 +310,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -592,7 +626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D17459BD-C9E4-7B4D-92D3-0201FF3B88CB}">
-  <dimension ref="A2:N58"/>
+  <dimension ref="A2:N57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="41" customWidth="1"/>
@@ -601,64 +635,69 @@
   <sheetData>
     <row r="2" spans="1:14" ht="24" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C5" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C6" t="s">
-        <v>51</v>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="C7" s="6" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:14" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>13</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:14" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C10" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="D12" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F12" t="s">
+        <v>61</v>
+      </c>
+      <c r="G12" t="s">
         <v>2</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>3</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>4</v>
       </c>
-      <c r="I12" t="s">
-        <v>5</v>
-      </c>
       <c r="J12" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="K12" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="N12" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
@@ -671,223 +710,316 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C14" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C15" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C18" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C20" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C21" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C18" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C19" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C20" s="2" t="s">
+      <c r="F21" s="1"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C23" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C25" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>17</v>
+      </c>
+      <c r="C27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F27" s="6">
+        <v>2.6</v>
+      </c>
+      <c r="G27" s="6">
+        <v>2</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C28" t="s">
+        <v>19</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G28" s="6">
+        <v>0</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C29" t="s">
+        <v>20</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="G29" s="6">
+        <v>0</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C30" t="s">
+        <v>21</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G30" s="6">
+        <v>0</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C31" t="s">
+        <v>20</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G31" s="6">
+        <v>0</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C32" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>23</v>
+      </c>
+      <c r="C34" t="s">
+        <v>24</v>
+      </c>
+      <c r="D34" t="s">
+        <v>40</v>
+      </c>
+      <c r="F34" t="s">
+        <v>58</v>
+      </c>
+      <c r="G34" s="6"/>
+      <c r="H34" s="6"/>
+      <c r="N34" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="C35" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D35" t="s">
+        <v>40</v>
+      </c>
+      <c r="G35" s="6"/>
+      <c r="H35" s="6"/>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="C36" t="s">
+        <v>24</v>
+      </c>
+      <c r="D36" t="s">
+        <v>41</v>
+      </c>
+      <c r="F36" t="s">
+        <v>58</v>
+      </c>
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+      <c r="N36" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="C37" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D37" t="s">
+        <v>41</v>
+      </c>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>26</v>
+      </c>
+      <c r="C39" t="s">
+        <v>27</v>
+      </c>
+      <c r="G39" s="6"/>
+      <c r="H39" s="6"/>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="C40" t="s">
+        <v>28</v>
+      </c>
+      <c r="G40" s="6"/>
+      <c r="H40" s="6"/>
+    </row>
+    <row r="43" spans="1:14" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C21" t="s">
-        <v>11</v>
-      </c>
-      <c r="F21" s="1"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C23" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C24" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C25" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>19</v>
-      </c>
-      <c r="C27" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C28" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C29" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C30" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C31" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C32" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="C33" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>26</v>
-      </c>
-      <c r="C35" t="s">
-        <v>27</v>
-      </c>
-      <c r="D35" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="C36" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D36" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="C37" t="s">
-        <v>27</v>
-      </c>
-      <c r="D37" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="C38" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D38" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
-        <v>29</v>
-      </c>
-      <c r="C40" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="C41" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="4" t="s">
+      <c r="C43" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="C44" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C44" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="45" spans="1:14" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C45" s="5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="46" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:14" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C46" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C47" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>32</v>
-      </c>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>29</v>
+      </c>
+      <c r="C48" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="49" spans="3:8" x14ac:dyDescent="0.2">
       <c r="C49" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="C50" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="C51" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="50" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C50" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="51" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C51" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="52" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C52" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="C52" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="C53" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="F52" s="6"/>
+      <c r="G52" s="6"/>
+      <c r="H52" s="6"/>
+    </row>
+    <row r="54" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C54" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D54" t="s">
+        <v>40</v>
+      </c>
+      <c r="G54" s="6"/>
+      <c r="H54" s="6"/>
+    </row>
+    <row r="55" spans="3:8" x14ac:dyDescent="0.2">
       <c r="C55" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D55" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+        <v>40</v>
+      </c>
+      <c r="G55" s="6"/>
+      <c r="H55" s="6"/>
+    </row>
+    <row r="56" spans="3:8" x14ac:dyDescent="0.2">
       <c r="C56" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D56" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+        <v>41</v>
+      </c>
+      <c r="G56" s="6"/>
+      <c r="H56" s="6"/>
+    </row>
+    <row r="57" spans="3:8" x14ac:dyDescent="0.2">
       <c r="C57" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D57" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="C58" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D58" t="s">
-        <v>44</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="G57" s="6"/>
+      <c r="H57" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
hw report updated + gitignore
</commit_message>
<xml_diff>
--- a/2_Assessments/Measurement_Table_Template.xlsx
+++ b/2_Assessments/Measurement_Table_Template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1185AC18-9611-445E-BE0E-EB15C61C57E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06F8D03D-0ECF-4B86-BFC6-08B5A6E8DE36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{4F5E00DF-9948-D646-B558-8B1F78610CF0}"/>
   </bookViews>
@@ -11,7 +11,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -32,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="115">
   <si>
     <t>Voltages</t>
   </si>
@@ -193,18 +192,9 @@
     <t>&amp; Currents</t>
   </si>
   <si>
-    <t>Voltage at +5V USB power</t>
-  </si>
-  <si>
     <t>light blue = additional measurements (optional)</t>
   </si>
   <si>
-    <t>4.75 V</t>
-  </si>
-  <si>
-    <t>5.25 V</t>
-  </si>
-  <si>
     <t>3.25 V</t>
   </si>
   <si>
@@ -277,9 +267,6 @@
     <t>0.8 uV RMS + 50 dB below the input (Lab Power Supply)</t>
   </si>
   <si>
-    <t>uVpp</t>
-  </si>
-  <si>
     <t>Keysight U3402A</t>
   </si>
   <si>
@@ -358,12 +345,6 @@
     <t>2.489V</t>
   </si>
   <si>
-    <t>2.55V</t>
-  </si>
-  <si>
-    <t>2.45V</t>
-  </si>
-  <si>
     <t>+- 2% (2 R)</t>
   </si>
   <si>
@@ -386,6 +367,15 @@
   </si>
   <si>
     <t>Sample rate</t>
+  </si>
+  <si>
+    <t>uV</t>
+  </si>
+  <si>
+    <t>2.475V</t>
+  </si>
+  <si>
+    <t>2.525V</t>
   </si>
 </sst>
 </file>
@@ -395,7 +385,7 @@
   <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0.000_-;\-* #,##0.000_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="169" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -504,7 +494,7 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -530,29 +520,14 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -565,8 +540,16 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="3" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -904,7 +887,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D17459BD-C9E4-7B4D-92D3-0201FF3B88CB}">
-  <dimension ref="A2:S61"/>
+  <dimension ref="A2:S60"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="3" max="3" width="41" customWidth="1"/>
@@ -945,7 +928,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.4">
       <c r="C8" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.4">
@@ -975,11 +958,11 @@
       <c r="D13" t="s">
         <v>35</v>
       </c>
-      <c r="F13" s="13" t="s">
+      <c r="F13" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22"/>
       <c r="I13" s="6" t="s">
         <v>2</v>
       </c>
@@ -1001,56 +984,62 @@
         <v>0</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="G14" s="11">
-        <v>5</v>
-      </c>
-      <c r="H14" s="11" t="s">
-        <v>72</v>
+        <v>56</v>
+      </c>
+      <c r="G14" s="6">
+        <v>3.3</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>69</v>
       </c>
       <c r="I14" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="J14" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="J14" s="6" t="s">
-        <v>56</v>
+      <c r="K14" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="L14" s="17" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="10" t="s">
-        <v>59</v>
+      <c r="C15" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="G15" s="6">
         <v>3.3</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="K15" s="24" t="s">
-        <v>100</v>
-      </c>
-      <c r="L15" s="22" t="s">
-        <v>82</v>
+        <v>55</v>
+      </c>
+      <c r="K15" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="L15" s="17" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.4">
       <c r="C16" s="1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G16" s="6">
-        <v>3.3</v>
+        <v>5</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I16" s="6" t="s">
         <v>57</v>
@@ -1058,121 +1047,131 @@
       <c r="J16" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="K16" s="24" t="s">
-        <v>83</v>
-      </c>
-      <c r="L16" s="22" t="s">
-        <v>82</v>
+      <c r="K16" s="19" t="s">
+        <v>93</v>
+      </c>
+      <c r="L16" s="17" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.4">
       <c r="C17" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G17" s="12">
+        <v>5.35</v>
+      </c>
+      <c r="H17" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="I17" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="J17" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="K17" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="L17" s="17" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="C18" t="s">
+        <v>7</v>
+      </c>
+      <c r="G18" s="12">
         <v>5</v>
       </c>
-      <c r="G17" s="6">
-        <v>5</v>
-      </c>
-      <c r="H17" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="J17" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="K17" s="24" t="s">
-        <v>97</v>
-      </c>
-      <c r="L17" s="22" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="C18" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="G18" s="12">
-        <v>5.35</v>
-      </c>
       <c r="H18" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="I18" s="12" t="s">
-        <v>95</v>
-      </c>
-      <c r="J18" s="12" t="s">
-        <v>96</v>
-      </c>
-      <c r="K18" s="25" t="s">
-        <v>84</v>
-      </c>
-      <c r="L18" s="22" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="C19" t="s">
-        <v>7</v>
-      </c>
-      <c r="G19" s="12">
-        <v>5</v>
-      </c>
-      <c r="H19" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
-      <c r="K19" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="L19" s="22" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="C21" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="F21" t="s">
-        <v>73</v>
-      </c>
-      <c r="G21" s="14">
+        <v>69</v>
+      </c>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="L18" s="17" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="C20" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="F20" t="s">
+        <v>70</v>
+      </c>
+      <c r="G20" s="13">
         <f>(0.8*(10^-6)+(1*10^-3)*(10^-5)/20)*10^6</f>
         <v>0.80049999999999999</v>
       </c>
-      <c r="H21" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="I21" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="J21" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="K21" s="25" t="s">
-        <v>87</v>
+      <c r="H20" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="I20" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="J20" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="K20" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="N20" t="s">
+        <v>77</v>
+      </c>
+      <c r="S20" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="C21" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F21" t="s">
+        <v>70</v>
+      </c>
+      <c r="G21" s="13">
+        <f>(0.8*(10^-6)+(1*10^-3)*(10^-5)/20)*10^6</f>
+        <v>0.80049999999999999</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="I21" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="K21" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="L21" s="17" t="s">
+        <v>90</v>
       </c>
       <c r="N21" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="S21" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.4">
       <c r="C22" s="1" t="s">
-        <v>6</v>
+        <v>85</v>
       </c>
       <c r="F22" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="G22" s="14">
-        <f>(0.8*(10^-6)+(1*10^-3)*(10^-5)/20)*10^6</f>
-        <v>0.80049999999999999</v>
-      </c>
-      <c r="H22" s="15" t="s">
-        <v>81</v>
+        <f>(0.8*10^-6+(G24*10^-3)*(10^-5)/20)*10^6</f>
+        <v>0.80499999999999994</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>112</v>
       </c>
       <c r="I22" s="9" t="s">
         <v>51</v>
@@ -1180,113 +1179,106 @@
       <c r="J22" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="K22" s="25" t="s">
+      <c r="K22" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="L22" s="22" t="s">
-        <v>94</v>
+      <c r="L22" s="17" t="s">
+        <v>90</v>
       </c>
       <c r="N22" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="S22" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.4">
       <c r="C23" s="1" t="s">
-        <v>89</v>
+        <v>9</v>
       </c>
       <c r="F23" t="s">
-        <v>73</v>
-      </c>
-      <c r="G23" s="16">
-        <f>(0.8*(10^-6)+G25*(10^-5)/20)*10^6</f>
-        <v>5.8</v>
-      </c>
-      <c r="H23" s="17" t="s">
-        <v>81</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
       <c r="I23" s="9" t="s">
         <v>51</v>
       </c>
       <c r="J23" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="K23" s="25" t="s">
+      <c r="K23" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="L23" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="L23" s="22" t="s">
-        <v>94</v>
-      </c>
-      <c r="N23" t="s">
-        <v>79</v>
-      </c>
-      <c r="S23" t="s">
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="C24" t="s">
+        <v>8</v>
+      </c>
+      <c r="F24" t="s">
+        <v>70</v>
+      </c>
+      <c r="G24" s="15">
+        <f>(1*(1-(5*0.9/G18))/((1*10^6)*(10*10^-6)))*10^3</f>
+        <v>9.9999999999999982</v>
+      </c>
+      <c r="H24" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="I24" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="J24" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="K24" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="L24" s="17" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="C26" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="G26" s="8">
+        <v>180</v>
+      </c>
+      <c r="H26" s="8" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="C24" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F24" t="s">
-        <v>73</v>
-      </c>
-      <c r="G24" s="12"/>
-      <c r="H24" s="12"/>
-      <c r="I24" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="J24" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="K24" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="L24" s="22" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="C25" t="s">
-        <v>8</v>
-      </c>
-      <c r="F25" t="s">
-        <v>73</v>
-      </c>
-      <c r="G25" s="18">
-        <f>(1*(1-(5*0.9/G19))/((1*10^6)*(10*10^-6)))*10^3</f>
-        <v>9.9999999999999982</v>
-      </c>
-      <c r="H25" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="I25" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="J25" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="K25" s="24" t="s">
+      <c r="I26" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="J26" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="K26" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="L25" s="22" t="s">
-        <v>94</v>
+      <c r="L26" s="17" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.4">
       <c r="C27" s="1" t="s">
-        <v>13</v>
+        <v>59</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="G27" s="8">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="I27" s="9" t="s">
         <v>51</v>
@@ -1294,302 +1286,294 @@
       <c r="J27" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="K27" s="24" t="s">
-        <v>92</v>
-      </c>
-      <c r="L27" s="22" t="s">
-        <v>82</v>
+      <c r="K27" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="L27" s="17" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="C28" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="G28" s="8">
-        <v>160</v>
-      </c>
-      <c r="H28" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="I28" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="J28" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="K28" s="24" t="s">
-        <v>93</v>
-      </c>
-      <c r="L28" s="22" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="C29" t="s">
+      <c r="C28" t="s">
         <v>49</v>
       </c>
-      <c r="F29" s="23"/>
-      <c r="G29" s="12"/>
-      <c r="H29" s="12"/>
-      <c r="I29" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="J29" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="K29" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="L29" s="22" t="s">
-        <v>99</v>
+      <c r="F28" s="18"/>
+      <c r="G28" s="12"/>
+      <c r="H28" s="12"/>
+      <c r="I28" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="J28" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="L28" s="17" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A30" t="s">
+        <v>14</v>
+      </c>
+      <c r="C30" t="s">
+        <v>15</v>
+      </c>
+      <c r="F30" s="5"/>
+      <c r="G30" s="8">
+        <v>2.6</v>
+      </c>
+      <c r="H30" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="I30" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="J30" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="K30" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="L30" s="17" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="A31" t="s">
-        <v>14</v>
-      </c>
       <c r="C31" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F31" s="5"/>
       <c r="G31" s="8">
-        <v>2.6</v>
+        <v>50</v>
       </c>
       <c r="H31" s="8" t="s">
         <v>72</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="J31" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="K31" s="24" t="s">
-        <v>101</v>
-      </c>
-      <c r="L31" s="22" t="s">
-        <v>82</v>
+        <v>46</v>
+      </c>
+      <c r="K31" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="L31" s="17" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.4">
       <c r="C32" t="s">
-        <v>16</v>
-      </c>
-      <c r="F32" s="5"/>
+        <v>17</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>73</v>
+      </c>
       <c r="G32" s="8">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I32" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J32" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="K32" s="24" t="s">
-        <v>102</v>
-      </c>
-      <c r="L32" s="22" t="s">
-        <v>94</v>
+      <c r="K32" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="L32" s="17" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.4">
       <c r="C33" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="G33" s="8">
-        <v>300</v>
+        <v>2</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J33" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="K33" s="24" t="s">
-        <v>103</v>
-      </c>
-      <c r="L33" s="22" t="s">
-        <v>94</v>
+      <c r="K33" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="L33" s="17" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.4">
       <c r="C34" t="s">
-        <v>18</v>
+        <v>102</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="G34" s="8">
         <v>2</v>
       </c>
       <c r="H34" s="8" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I34" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J34" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="K34" s="24" t="s">
-        <v>104</v>
-      </c>
-      <c r="L34" s="22" t="s">
-        <v>94</v>
+      <c r="K34" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="L34" s="17" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.4">
       <c r="C35" t="s">
-        <v>106</v>
-      </c>
-      <c r="F35" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="G35" s="8">
-        <v>2</v>
-      </c>
-      <c r="H35" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="I35" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="J35" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="K35" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="G35" s="6">
+        <v>2.5</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="K35" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="L35" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="N35" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="L35" s="22" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="C36" t="s">
-        <v>19</v>
-      </c>
-      <c r="F36" s="26"/>
-      <c r="G36" s="15">
-        <v>2.5</v>
-      </c>
-      <c r="H36" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="I36" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="J36" s="15" t="s">
-        <v>108</v>
-      </c>
-      <c r="K36" s="24" t="s">
-        <v>107</v>
-      </c>
-      <c r="L36" s="22" t="s">
-        <v>82</v>
-      </c>
-      <c r="N36" s="27" t="s">
-        <v>110</v>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="A37" t="s">
+        <v>20</v>
+      </c>
+      <c r="C37" t="s">
+        <v>21</v>
+      </c>
+      <c r="D37" t="s">
+        <v>36</v>
+      </c>
+      <c r="G37" s="6">
+        <v>500</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="I37" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="J37" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="N37" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A38" t="s">
-        <v>20</v>
-      </c>
-      <c r="C38" t="s">
-        <v>21</v>
+      <c r="C38" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="D38" t="s">
         <v>36</v>
       </c>
-      <c r="G38" s="6">
+      <c r="G38" s="12"/>
+      <c r="H38" s="12"/>
+      <c r="I38" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="J38" s="9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="C39" t="s">
+        <v>21</v>
+      </c>
+      <c r="D39" t="s">
+        <v>37</v>
+      </c>
+      <c r="G39" s="6">
         <v>500</v>
       </c>
-      <c r="H38" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="I38" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="J38" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="N38" t="s">
+      <c r="H39" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="I39" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="J39" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="N39" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="C39" s="1" t="s">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="C40" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="D39" t="s">
-        <v>36</v>
-      </c>
-      <c r="G39" s="12"/>
-      <c r="H39" s="12"/>
-      <c r="I39" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="J39" s="9" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="C40" t="s">
-        <v>21</v>
       </c>
       <c r="D40" t="s">
         <v>37</v>
       </c>
-      <c r="G40" s="6">
-        <v>500</v>
-      </c>
-      <c r="H40" s="6" t="s">
-        <v>77</v>
-      </c>
+      <c r="G40" s="12"/>
+      <c r="H40" s="12"/>
       <c r="I40" s="9" t="s">
         <v>51</v>
       </c>
       <c r="J40" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="N40" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="C41" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D41" t="s">
-        <v>37</v>
-      </c>
-      <c r="G41" s="12"/>
-      <c r="H41" s="12"/>
-      <c r="I41" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="J41" s="9" t="s">
-        <v>51</v>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="A42" t="s">
+        <v>23</v>
+      </c>
+      <c r="C42" t="s">
+        <v>24</v>
+      </c>
+      <c r="G42" s="12"/>
+      <c r="H42" s="12"/>
+      <c r="I42" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="J42" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="K42" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="L42" s="17" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A43" t="s">
-        <v>23</v>
-      </c>
       <c r="C43" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G43" s="12"/>
       <c r="H43" s="12"/>
@@ -1600,37 +1584,28 @@
         <v>51</v>
       </c>
       <c r="K43" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="L43" s="22" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="C44" t="s">
-        <v>25</v>
-      </c>
-      <c r="G44" s="12"/>
-      <c r="H44" s="12"/>
-      <c r="I44" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="J44" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="K44" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="L44" s="22" t="s">
-        <v>82</v>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="L43" s="17" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A46" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G46" s="7"/>
+      <c r="H46" s="7"/>
+      <c r="I46" s="7"/>
+      <c r="J46" s="7"/>
+      <c r="K46" s="7"/>
     </row>
     <row r="47" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="A47" s="3" t="s">
-        <v>10</v>
-      </c>
       <c r="C47" s="4" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G47" s="7"/>
       <c r="H47" s="7"/>
@@ -1640,7 +1615,7 @@
     </row>
     <row r="48" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.4">
       <c r="C48" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G48" s="7"/>
       <c r="H48" s="7"/>
@@ -1650,7 +1625,7 @@
     </row>
     <row r="49" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.4">
       <c r="C49" s="4" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="G49" s="7"/>
       <c r="H49" s="7"/>
@@ -1658,124 +1633,130 @@
       <c r="J49" s="7"/>
       <c r="K49" s="7"/>
     </row>
-    <row r="50" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="C50" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="G50" s="7"/>
-      <c r="H50" s="7"/>
-      <c r="I50" s="7"/>
-      <c r="J50" s="7"/>
-      <c r="K50" s="7"/>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="A51" t="s">
+        <v>26</v>
+      </c>
+      <c r="C51" t="s">
+        <v>41</v>
+      </c>
+      <c r="F51" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="G51" s="23"/>
+      <c r="H51" s="23"/>
+      <c r="I51" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="J51" s="6" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A52" t="s">
-        <v>26</v>
-      </c>
       <c r="C52" t="s">
-        <v>41</v>
-      </c>
-      <c r="F52" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="G52" s="20"/>
-      <c r="H52" s="20"/>
+        <v>38</v>
+      </c>
+      <c r="F52" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="G52" s="23"/>
+      <c r="H52" s="23"/>
       <c r="I52" s="6" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="J52" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="K52" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L52" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="N52" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="C53" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F53" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="G53" s="23"/>
+      <c r="H53" s="23"/>
+      <c r="I53" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="J53" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="K53" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="L53" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="N53" s="6" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="C54" t="s">
+        <v>40</v>
+      </c>
+      <c r="F54" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="C53" t="s">
-        <v>38</v>
-      </c>
-      <c r="F53" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="G53" s="20"/>
-      <c r="H53" s="20"/>
-      <c r="I53" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="J53" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K53" s="24" t="s">
-        <v>113</v>
-      </c>
-      <c r="L53" s="22" t="s">
-        <v>94</v>
-      </c>
-      <c r="N53" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="C54" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F54" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="G54" s="20"/>
-      <c r="H54" s="20"/>
-      <c r="I54" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="J54" s="15" t="s">
-        <v>116</v>
-      </c>
-      <c r="K54" s="24" t="s">
-        <v>114</v>
-      </c>
-      <c r="L54" s="22" t="s">
-        <v>94</v>
-      </c>
-      <c r="N54" s="6" t="s">
-        <v>117</v>
+      <c r="G54" s="11">
+        <v>100</v>
+      </c>
+      <c r="H54" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="I54" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="J54" s="11" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.4">
       <c r="C55" t="s">
-        <v>40</v>
-      </c>
-      <c r="F55" t="s">
-        <v>73</v>
-      </c>
-      <c r="G55" s="11">
-        <v>100</v>
-      </c>
-      <c r="H55" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="I55" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="J55" s="11" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="C56" t="s">
         <v>42</v>
       </c>
-      <c r="F56" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="G56" s="21"/>
-      <c r="H56" s="21"/>
-      <c r="I56" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="J56" s="9" t="s">
+      <c r="F55" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="G55" s="24"/>
+      <c r="H55" s="24"/>
+      <c r="I55" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="J55" s="9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="C57" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D57" t="s">
+        <v>36</v>
+      </c>
+      <c r="G57" s="12"/>
+      <c r="H57" s="12"/>
+      <c r="I57" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="J57" s="9" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.4">
       <c r="C58" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D58" t="s">
         <v>36</v>
@@ -1791,10 +1772,10 @@
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.4">
       <c r="C59" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D59" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G59" s="12"/>
       <c r="H59" s="12"/>
@@ -1807,7 +1788,7 @@
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.4">
       <c r="C60" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D60" t="s">
         <v>37</v>
@@ -1821,29 +1802,13 @@
         <v>51</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="C61" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D61" t="s">
-        <v>37</v>
-      </c>
-      <c r="G61" s="12"/>
-      <c r="H61" s="12"/>
-      <c r="I61" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="J61" s="9" t="s">
-        <v>51</v>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="F13:H13"/>
+    <mergeCell ref="F51:H51"/>
     <mergeCell ref="F52:H52"/>
+    <mergeCell ref="F55:H55"/>
     <mergeCell ref="F53:H53"/>
-    <mergeCell ref="F56:H56"/>
-    <mergeCell ref="F54:H54"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
hw report some more wip
</commit_message>
<xml_diff>
--- a/2_Assessments/Measurement_Table_Template.xlsx
+++ b/2_Assessments/Measurement_Table_Template.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B37D0ABA-F0EF-45D0-9DB7-A232F7E8938F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BC3417D-451A-4E76-A76E-8121B0EBB0FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{4F5E00DF-9948-D646-B558-8B1F78610CF0}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{4F5E00DF-9948-D646-B558-8B1F78610CF0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="116">
   <si>
     <t>Voltages</t>
   </si>
@@ -373,6 +373,12 @@
   </si>
   <si>
     <t>2.525V</t>
+  </si>
+  <si>
+    <t>1.2Vpp</t>
+  </si>
+  <si>
+    <t>1kHz is in pass band =&gt; no attenuation</t>
   </si>
 </sst>
 </file>
@@ -1116,6 +1122,9 @@
       <c r="K20" s="20" t="s">
         <v>83</v>
       </c>
+      <c r="L20" s="17" t="s">
+        <v>90</v>
+      </c>
       <c r="N20" t="s">
         <v>77</v>
       </c>
@@ -1485,6 +1494,10 @@
       <c r="J37" s="9" t="s">
         <v>51</v>
       </c>
+      <c r="K37" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="L37" s="11"/>
       <c r="N37" t="s">
         <v>47</v>
       </c>
@@ -1496,13 +1509,26 @@
       <c r="D38" t="s">
         <v>36</v>
       </c>
-      <c r="G38" s="12"/>
-      <c r="H38" s="12"/>
+      <c r="G38" s="6">
+        <v>500</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>74</v>
+      </c>
       <c r="I38" s="9" t="s">
         <v>51</v>
       </c>
       <c r="J38" s="9" t="s">
         <v>51</v>
+      </c>
+      <c r="K38" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="L38" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="N38" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.4">
@@ -1524,6 +1550,10 @@
       <c r="J39" s="9" t="s">
         <v>51</v>
       </c>
+      <c r="K39" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="L39" s="11"/>
       <c r="N39" t="s">
         <v>47</v>
       </c>
@@ -1535,13 +1565,26 @@
       <c r="D40" t="s">
         <v>37</v>
       </c>
-      <c r="G40" s="12"/>
-      <c r="H40" s="12"/>
+      <c r="G40" s="6">
+        <v>500</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>74</v>
+      </c>
       <c r="I40" s="9" t="s">
         <v>51</v>
       </c>
       <c r="J40" s="9" t="s">
         <v>51</v>
+      </c>
+      <c r="K40" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="L40" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="N40" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.4">

</xml_diff>